<commit_message>
Add decision report and market-aware strike selection
</commit_message>
<xml_diff>
--- a/exports/earnings_test_2026-07-14.xlsx
+++ b/exports/earnings_test_2026-07-14.xlsx
@@ -480,7 +480,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12.89999961853027</v>
+        <v>13</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -488,28 +488,28 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>-3.100772328362644</v>
+        <v>-23.07692307692307</v>
       </c>
       <c r="E2" t="n">
-        <v>-22.48061786269011</v>
+        <v>-42.30769230769231</v>
       </c>
       <c r="F2" t="n">
-        <v>-3.100772328362644</v>
+        <v>15.38461538461537</v>
       </c>
       <c r="G2" t="n">
-        <v>16.27907320596482</v>
+        <v>34.61538461538463</v>
       </c>
       <c r="H2" t="n">
-        <v>12.5</v>
+        <v>10</v>
       </c>
       <c r="I2" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="J2" t="n">
-        <v>12.5</v>
+        <v>15</v>
       </c>
       <c r="K2" t="n">
-        <v>15</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="3">
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>59.34000015258789</v>
+        <v>60.61999893188477</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -527,22 +527,22 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-3.100775442966774</v>
+        <v>-2.672383636471298</v>
       </c>
       <c r="E3" t="n">
-        <v>-11.52679496966531</v>
+        <v>-10.92048671812628</v>
       </c>
       <c r="F3" t="n">
-        <v>4.482642131061909</v>
+        <v>2.276478212521682</v>
       </c>
       <c r="G3" t="n">
-        <v>12.90866165776046</v>
+        <v>10.52458129417666</v>
       </c>
       <c r="H3" t="n">
-        <v>57.5</v>
+        <v>59</v>
       </c>
       <c r="I3" t="n">
-        <v>52.5</v>
+        <v>54</v>
       </c>
       <c r="J3" t="n">
         <v>62</v>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>138.6399993896484</v>
+        <v>133.2700042724609</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -566,28 +566,28 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-4.789382154414678</v>
+        <v>-3.954381408802832</v>
       </c>
       <c r="E4" t="n">
-        <v>-8.395844951595944</v>
+        <v>-7.706163385021469</v>
       </c>
       <c r="F4" t="n">
-        <v>4.587421118256607</v>
+        <v>5.049895334121901</v>
       </c>
       <c r="G4" t="n">
-        <v>8.193883915437873</v>
+        <v>8.801677310340539</v>
       </c>
       <c r="H4" t="n">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I4" t="n">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="J4" t="n">
+        <v>140</v>
+      </c>
+      <c r="K4" t="n">
         <v>145</v>
-      </c>
-      <c r="K4" t="n">
-        <v>150</v>
       </c>
     </row>
     <row r="5">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11.60970020294189</v>
+        <v>10.14000034332275</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -605,28 +605,28 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>-5.251644678881517</v>
+        <v>-11.24260655546674</v>
       </c>
       <c r="E5" t="n">
-        <v>-31.09210522100474</v>
+        <v>-40.82840437031115</v>
       </c>
       <c r="F5" t="n">
-        <v>3.36184216849289</v>
+        <v>8.481258654429546</v>
       </c>
       <c r="G5" t="n">
-        <v>20.58881586324171</v>
+        <v>28.20512386432581</v>
       </c>
       <c r="H5" t="n">
+        <v>9</v>
+      </c>
+      <c r="I5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J5" t="n">
         <v>11</v>
       </c>
-      <c r="I5" t="n">
-        <v>8</v>
-      </c>
-      <c r="J5" t="n">
-        <v>12</v>
-      </c>
       <c r="K5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -636,7 +636,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46.90499877929688</v>
+        <v>45.7400016784668</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -644,16 +644,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>-9.391320528594004</v>
+        <v>-7.083518932165022</v>
       </c>
       <c r="E6" t="n">
-        <v>-14.72124285044142</v>
+        <v>-12.5491942890965</v>
       </c>
       <c r="F6" t="n">
-        <v>1.268524115100811</v>
+        <v>3.847831781697919</v>
       </c>
       <c r="G6" t="n">
-        <v>6.598446436948224</v>
+        <v>9.313507138629372</v>
       </c>
       <c r="H6" t="n">
         <v>42.5</v>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1041.089965820312</v>
+        <v>1140</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -683,28 +683,28 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>-4.907353590720365</v>
+        <v>-3.508771929824561</v>
       </c>
       <c r="E7" t="n">
-        <v>-6.828417154544198</v>
+        <v>-5.263157894736848</v>
       </c>
       <c r="F7" t="n">
-        <v>5.178230119354743</v>
+        <v>3.947368421052633</v>
       </c>
       <c r="G7" t="n">
-        <v>7.099293683178587</v>
+        <v>5.701754385964919</v>
       </c>
       <c r="H7" t="n">
-        <v>990</v>
+        <v>1100</v>
       </c>
       <c r="I7" t="n">
-        <v>970</v>
+        <v>1080</v>
       </c>
       <c r="J7" t="n">
-        <v>1095</v>
+        <v>1185</v>
       </c>
       <c r="K7" t="n">
-        <v>1115</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="8">
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>334.7780151367188</v>
+        <v>342.8900146484375</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -722,28 +722,28 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>-4.414272881892678</v>
+        <v>-3.030130422167676</v>
       </c>
       <c r="E8" t="n">
-        <v>-10.38838082677439</v>
+        <v>-8.862904532112481</v>
       </c>
       <c r="F8" t="n">
-        <v>4.54688903542988</v>
+        <v>3.531740451520227</v>
       </c>
       <c r="G8" t="n">
-        <v>10.52099698031159</v>
+        <v>9.364514561465032</v>
       </c>
       <c r="H8" t="n">
-        <v>320</v>
+        <v>332.5</v>
       </c>
       <c r="I8" t="n">
-        <v>300</v>
+        <v>312.5</v>
       </c>
       <c r="J8" t="n">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="K8" t="n">
-        <v>370</v>
+        <v>375</v>
       </c>
     </row>
     <row r="9">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>86.87000274658203</v>
+        <v>85.29000091552734</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -761,28 +761,28 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>-5.606081032124344</v>
+        <v>-2.684958249438174</v>
       </c>
       <c r="E9" t="n">
-        <v>-11.36180779845822</v>
+        <v>-8.547310162122624</v>
       </c>
       <c r="F9" t="n">
-        <v>4.754227147276646</v>
+        <v>5.522334428320064</v>
       </c>
       <c r="G9" t="n">
-        <v>10.50995391361051</v>
+        <v>11.38468634100451</v>
       </c>
       <c r="H9" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I9" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J9" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="K9" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>